<commit_message>
Corrige K/D total para kills÷deaths em vez da média por partida.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/Estatisticas_CS2.xlsx
+++ b/data/Estatisticas_CS2.xlsx
@@ -1,21 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados_Por_Partida" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totais_e_Medias_Gerais" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties">
+  <dc:creator xmlns:dc="http://purl.org/dc/elements/1.1/">openpyxl</dc:creator>
+  <dcterms:created xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-12T01:31:08Z</dcterms:created>
+  <dcterms:modified xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xsi:type="dcterms:W3CDTF">2026-07-12T01:37:16Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="3">
@@ -167,7 +166,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -450,7 +449,23 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados_Por_Partida" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totais_e_Medias_Gerais" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1638,7 +1653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1709,7 +1724,7 @@
         <v>94</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1.117142857142857</v>
+        <v>0.9574468085106383</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>74.14285714285714</v>
@@ -1734,7 +1749,7 @@
         <v>85</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.142857142857143</v>
+        <v>1.2588235294117647</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>84.57142857142857</v>
@@ -1759,7 +1774,7 @@
         <v>88</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1.052857142857143</v>
+        <v>1.125</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>66</v>
@@ -1784,7 +1799,7 @@
         <v>83</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1.565714285714286</v>
+        <v>1.253012048192771</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>83.57142857142857</v>
@@ -1809,7 +1824,7 @@
         <v>89</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1.13</v>
+        <v>0.8314606741573034</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>55.57142857142857</v>

</xml_diff>